<commit_message>
section 4.2 base case input param corrected
</commit_message>
<xml_diff>
--- a/Section 4.2/Data_section4.2.xlsx
+++ b/Section 4.2/Data_section4.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KUNTEAM\Documents\GitHub\Physics-informed-multiscale-optimization-of-renewable-powered-alkaline-water-electrolysis\Section 4.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A09CCCB-1A2D-4C01-BFAB-CCCF754FDE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAD02AB-676F-4BA1-B09F-7C4BABAF43E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{7C88D86B-F107-4116-B17D-B8DFC6C89132}"/>
+    <workbookView xWindow="8550" yWindow="2310" windowWidth="39780" windowHeight="17325" xr2:uid="{7C88D86B-F107-4116-B17D-B8DFC6C89132}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +144,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -165,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -173,6 +184,8 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -517,7 +530,7 @@
     <col min="12" max="12" width="12.5703125" customWidth="1"/>
     <col min="13" max="13" width="14.140625" customWidth="1"/>
     <col min="15" max="15" width="16.7109375" customWidth="1"/>
-    <col min="16" max="16" width="10.5703125" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" customWidth="1"/>
     <col min="17" max="17" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="21" customWidth="1"/>
     <col min="19" max="19" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -1447,32 +1460,32 @@
       <c r="M30">
         <v>1.6639999999999999</v>
       </c>
-      <c r="R30">
+      <c r="R30" s="5">
         <v>6.5</v>
       </c>
-      <c r="S30">
-        <v>4.6473899999999997</v>
-      </c>
-      <c r="T30">
-        <v>0.4</v>
-      </c>
-      <c r="U30">
-        <v>1.01936</v>
-      </c>
-      <c r="V30">
-        <v>0.75</v>
-      </c>
-      <c r="W30">
-        <v>2.2667700000000002</v>
-      </c>
-      <c r="X30">
-        <v>1.38253</v>
-      </c>
-      <c r="Y30">
-        <v>5.7563399999999998</v>
-      </c>
-      <c r="Z30">
-        <v>4.0199999999999996</v>
+      <c r="S30" s="5">
+        <v>4.6412340404969488</v>
+      </c>
+      <c r="T30" s="5">
+        <v>0.40000043468948587</v>
+      </c>
+      <c r="U30" s="5">
+        <v>1.0151367464074967</v>
+      </c>
+      <c r="V30" s="5">
+        <v>0.75001258065114207</v>
+      </c>
+      <c r="W30" s="5">
+        <v>2.0982174223388905</v>
+      </c>
+      <c r="X30" s="5">
+        <v>1.3878939002796704</v>
+      </c>
+      <c r="Y30" s="5">
+        <v>5.7421407736955761</v>
+      </c>
+      <c r="Z30" s="5">
+        <v>4.03</v>
       </c>
     </row>
     <row r="31" spans="5:27" x14ac:dyDescent="0.25">
@@ -1494,32 +1507,32 @@
       <c r="M31">
         <v>1.71075</v>
       </c>
-      <c r="R31">
+      <c r="R31" s="5">
         <v>8</v>
       </c>
-      <c r="S31">
-        <v>6.0746000000000002</v>
-      </c>
-      <c r="T31">
-        <v>0.52791999999999994</v>
-      </c>
-      <c r="U31">
-        <v>1.04541</v>
-      </c>
-      <c r="V31">
-        <v>0.75053000000000003</v>
-      </c>
-      <c r="W31">
-        <v>3.4791099999999999</v>
-      </c>
-      <c r="X31">
-        <v>0.51678000000000002</v>
-      </c>
-      <c r="Y31">
-        <v>10.74357</v>
-      </c>
-      <c r="Z31">
-        <v>3.82</v>
+      <c r="S31" s="5">
+        <v>5.7051387927969008</v>
+      </c>
+      <c r="T31" s="5">
+        <v>0.67792244742039498</v>
+      </c>
+      <c r="U31" s="5">
+        <v>1.0454328008672278</v>
+      </c>
+      <c r="V31" s="5">
+        <v>0.75679952167540654</v>
+      </c>
+      <c r="W31" s="5">
+        <v>5.0344711332363357</v>
+      </c>
+      <c r="X31" s="5">
+        <v>0.53153438267985442</v>
+      </c>
+      <c r="Y31" s="5">
+        <v>11.341731676860768</v>
+      </c>
+      <c r="Z31" s="5">
+        <v>3.81</v>
       </c>
     </row>
     <row r="32" spans="5:27" x14ac:dyDescent="0.25">
@@ -1541,31 +1554,31 @@
       <c r="M32">
         <v>1.7016</v>
       </c>
-      <c r="R32">
+      <c r="R32" s="5">
         <v>10</v>
       </c>
-      <c r="S32">
-        <v>6.5248200000000001</v>
-      </c>
-      <c r="T32">
-        <v>0.40360000000000001</v>
-      </c>
-      <c r="U32">
-        <v>1.1869499999999999</v>
-      </c>
-      <c r="V32">
-        <v>0.98014000000000001</v>
-      </c>
-      <c r="W32">
-        <v>3.25</v>
-      </c>
-      <c r="X32">
-        <v>0.42687000000000003</v>
-      </c>
-      <c r="Y32">
-        <v>10.690060000000001</v>
-      </c>
-      <c r="Z32">
+      <c r="S32" s="5">
+        <v>6.0938761869116673</v>
+      </c>
+      <c r="T32" s="5">
+        <v>0.41620636974480868</v>
+      </c>
+      <c r="U32" s="5">
+        <v>1.0722874911175864</v>
+      </c>
+      <c r="V32" s="5">
+        <v>1.0146670945118841</v>
+      </c>
+      <c r="W32" s="5">
+        <v>5.5538562236651288</v>
+      </c>
+      <c r="X32" s="5">
+        <v>0.41317497727173147</v>
+      </c>
+      <c r="Y32" s="5">
+        <v>10.81682356786026</v>
+      </c>
+      <c r="Z32" s="5">
         <v>3.97</v>
       </c>
     </row>
@@ -1588,32 +1601,32 @@
       <c r="M33">
         <v>1.76332</v>
       </c>
-      <c r="R33">
+      <c r="R33" s="5">
         <v>15</v>
       </c>
-      <c r="S33">
-        <v>6.7104600000000003</v>
-      </c>
-      <c r="T33">
-        <v>0.43896000000000002</v>
-      </c>
-      <c r="U33">
-        <v>2.24926</v>
-      </c>
-      <c r="V33">
-        <v>1.0974900000000001</v>
-      </c>
-      <c r="W33">
-        <v>2.71604</v>
-      </c>
-      <c r="X33">
-        <v>0.50622999999999996</v>
-      </c>
-      <c r="Y33">
-        <v>10.48334</v>
-      </c>
-      <c r="Z33">
-        <v>4.28</v>
+      <c r="S33" s="5">
+        <v>8.0592901592029804</v>
+      </c>
+      <c r="T33" s="5">
+        <v>0.4168931326714706</v>
+      </c>
+      <c r="U33" s="5">
+        <v>2.3024999811573608</v>
+      </c>
+      <c r="V33" s="5">
+        <v>1.0078128952395105</v>
+      </c>
+      <c r="W33" s="5">
+        <v>2.112769330305353</v>
+      </c>
+      <c r="X33" s="5">
+        <v>0.44317987274666654</v>
+      </c>
+      <c r="Y33" s="5">
+        <v>10.933675400172245</v>
+      </c>
+      <c r="Z33" s="5">
+        <v>4.29</v>
       </c>
     </row>
     <row r="34" spans="5:27" x14ac:dyDescent="0.25">
@@ -1635,32 +1648,32 @@
       <c r="M34">
         <v>1.72271</v>
       </c>
-      <c r="R34">
+      <c r="R34" s="5">
         <v>20</v>
       </c>
-      <c r="S34">
-        <v>6.7796000000000003</v>
-      </c>
-      <c r="T34">
-        <v>0.40006000000000003</v>
-      </c>
-      <c r="U34">
-        <v>3.3277700000000001</v>
-      </c>
-      <c r="V34">
-        <v>1.24759</v>
-      </c>
-      <c r="W34">
-        <v>2.3755899999999999</v>
-      </c>
-      <c r="X34">
-        <v>0.44774999999999998</v>
-      </c>
-      <c r="Y34">
-        <v>11.003259999999999</v>
-      </c>
-      <c r="Z34">
-        <v>4.5599999999999996</v>
+      <c r="S34" s="5">
+        <v>5.7468093028448672</v>
+      </c>
+      <c r="T34" s="5">
+        <v>0.40020119947760274</v>
+      </c>
+      <c r="U34" s="5">
+        <v>2.7633439239954671</v>
+      </c>
+      <c r="V34" s="5">
+        <v>1.6232021970520087</v>
+      </c>
+      <c r="W34" s="5">
+        <v>2.0331707369967931</v>
+      </c>
+      <c r="X34" s="5">
+        <v>0.37548204949649866</v>
+      </c>
+      <c r="Y34" s="5">
+        <v>11.735150136134466</v>
+      </c>
+      <c r="Z34" s="5">
+        <v>4.58</v>
       </c>
     </row>
     <row r="35" spans="5:27" x14ac:dyDescent="0.25">
@@ -1682,31 +1695,31 @@
       <c r="M35">
         <v>1.71496</v>
       </c>
-      <c r="R35">
+      <c r="R35" s="5">
         <v>25</v>
       </c>
-      <c r="S35">
-        <v>7.3887600000000004</v>
-      </c>
-      <c r="T35">
-        <v>0.40064</v>
-      </c>
-      <c r="U35">
-        <v>5.3582000000000001</v>
-      </c>
-      <c r="V35">
-        <v>1.18272</v>
-      </c>
-      <c r="W35">
-        <v>2.55199</v>
-      </c>
-      <c r="X35">
-        <v>0.43231000000000003</v>
-      </c>
-      <c r="Y35">
-        <v>11.21641</v>
-      </c>
-      <c r="Z35">
+      <c r="S35" s="5">
+        <v>7.7252306265020856</v>
+      </c>
+      <c r="T35" s="5">
+        <v>0.40167764657500132</v>
+      </c>
+      <c r="U35" s="5">
+        <v>5.3625194829293674</v>
+      </c>
+      <c r="V35" s="5">
+        <v>1.1355122844377952</v>
+      </c>
+      <c r="W35" s="5">
+        <v>3.1713424102657437</v>
+      </c>
+      <c r="X35" s="5">
+        <v>0.41822337008501853</v>
+      </c>
+      <c r="Y35" s="5">
+        <v>11.285256669389449</v>
+      </c>
+      <c r="Z35" s="5">
         <v>4.83</v>
       </c>
     </row>
@@ -1729,31 +1742,31 @@
       <c r="M36">
         <v>1.8164899999999999</v>
       </c>
-      <c r="R36">
+      <c r="R36" s="5">
         <v>28</v>
       </c>
-      <c r="S36">
-        <v>6.6465699999999996</v>
-      </c>
-      <c r="T36">
-        <v>0.40083999999999997</v>
-      </c>
-      <c r="U36">
-        <v>5.5630899999999999</v>
-      </c>
-      <c r="V36">
-        <v>1.4836800000000001</v>
-      </c>
-      <c r="W36">
-        <v>3.0613600000000001</v>
-      </c>
-      <c r="X36">
-        <v>0.39351999999999998</v>
-      </c>
-      <c r="Y36">
-        <v>11.40687</v>
-      </c>
-      <c r="Z36">
+      <c r="S36" s="6">
+        <v>6.685384218104172</v>
+      </c>
+      <c r="T36" s="6">
+        <v>0.40847521344729992</v>
+      </c>
+      <c r="U36" s="6">
+        <v>5.8800090718777822</v>
+      </c>
+      <c r="V36" s="6">
+        <v>1.3183009042803449</v>
+      </c>
+      <c r="W36" s="6">
+        <v>2.3873039730711709</v>
+      </c>
+      <c r="X36" s="6">
+        <v>0.41445629722515726</v>
+      </c>
+      <c r="Y36" s="6">
+        <v>11.419430167495724</v>
+      </c>
+      <c r="Z36" s="6">
         <v>4.84</v>
       </c>
     </row>
@@ -1776,31 +1789,31 @@
       <c r="M37">
         <v>1.7059200000000001</v>
       </c>
-      <c r="R37">
+      <c r="R37" s="5">
         <v>30</v>
       </c>
-      <c r="S37">
-        <v>6.0097699999999996</v>
-      </c>
-      <c r="T37">
-        <v>0.40038000000000001</v>
-      </c>
-      <c r="U37">
-        <v>5.72302</v>
-      </c>
-      <c r="V37">
-        <v>1.47967</v>
-      </c>
-      <c r="W37">
-        <v>2.9521799999999998</v>
-      </c>
-      <c r="X37">
-        <v>0.40382000000000001</v>
-      </c>
-      <c r="Y37">
-        <v>11.264379999999999</v>
-      </c>
-      <c r="Z37">
+      <c r="S37" s="5">
+        <v>6.0209794864724069</v>
+      </c>
+      <c r="T37" s="5">
+        <v>0.4004294421207964</v>
+      </c>
+      <c r="U37" s="5">
+        <v>5.537229305447374</v>
+      </c>
+      <c r="V37" s="5">
+        <v>1.5221593619433653</v>
+      </c>
+      <c r="W37" s="5">
+        <v>2.7161933322255534</v>
+      </c>
+      <c r="X37" s="5">
+        <v>0.38668588404180959</v>
+      </c>
+      <c r="Y37" s="5">
+        <v>11.523478696418266</v>
+      </c>
+      <c r="Z37" s="5">
         <v>4.96</v>
       </c>
     </row>
@@ -1823,32 +1836,32 @@
       <c r="M38">
         <v>1.7220599999999999</v>
       </c>
-      <c r="R38">
+      <c r="R38" s="5">
         <v>35</v>
       </c>
-      <c r="S38">
-        <v>6.2881099999999996</v>
-      </c>
-      <c r="T38">
-        <v>0.40455999999999998</v>
-      </c>
-      <c r="U38">
-        <v>7.8281299999999998</v>
-      </c>
-      <c r="V38">
-        <v>1.37812</v>
-      </c>
-      <c r="W38">
-        <v>3.15645</v>
-      </c>
-      <c r="X38">
-        <v>0.38240000000000002</v>
-      </c>
-      <c r="Y38">
-        <v>11.24784</v>
-      </c>
-      <c r="Z38">
-        <v>5.16</v>
+      <c r="S38" s="5">
+        <v>5.672737320648916</v>
+      </c>
+      <c r="T38" s="5">
+        <v>0.403250789051667</v>
+      </c>
+      <c r="U38" s="5">
+        <v>6.8554270686239853</v>
+      </c>
+      <c r="V38" s="5">
+        <v>1.6189855221017373</v>
+      </c>
+      <c r="W38" s="5">
+        <v>2.4674663903553467</v>
+      </c>
+      <c r="X38" s="5">
+        <v>0.37579419450851093</v>
+      </c>
+      <c r="Y38" s="5">
+        <v>11.416356026966099</v>
+      </c>
+      <c r="Z38" s="5">
+        <v>5.15</v>
       </c>
     </row>
     <row r="39" spans="5:27" x14ac:dyDescent="0.25">
@@ -1870,31 +1883,31 @@
       <c r="M39">
         <v>1.72763</v>
       </c>
-      <c r="R39">
+      <c r="R39" s="5">
         <v>40</v>
       </c>
-      <c r="S39">
-        <v>6.5821300000000003</v>
-      </c>
-      <c r="T39">
-        <v>0.40056000000000003</v>
-      </c>
-      <c r="U39">
-        <v>10.05129</v>
-      </c>
-      <c r="V39">
-        <v>1.2870999999999999</v>
-      </c>
-      <c r="W39">
-        <v>3.2674699999999999</v>
-      </c>
-      <c r="X39">
-        <v>0.37689</v>
-      </c>
-      <c r="Y39">
-        <v>11.02736</v>
-      </c>
-      <c r="Z39">
+      <c r="S39" s="5">
+        <v>4.7268655446548919</v>
+      </c>
+      <c r="T39" s="5">
+        <v>0.42920832656212443</v>
+      </c>
+      <c r="U39" s="5">
+        <v>6.750644508869482</v>
+      </c>
+      <c r="V39" s="5">
+        <v>1.8628564894808151</v>
+      </c>
+      <c r="W39" s="5">
+        <v>2.9074743735478301</v>
+      </c>
+      <c r="X39" s="5">
+        <v>0.37731080130379169</v>
+      </c>
+      <c r="Y39" s="5">
+        <v>11.164600893232834</v>
+      </c>
+      <c r="Z39" s="5">
         <v>5.2</v>
       </c>
     </row>
@@ -2083,7 +2096,7 @@
       <c r="Z48" s="3"/>
       <c r="AA48" s="3"/>
     </row>
-    <row r="49" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E49">
         <v>5.1244699999999996</v>
       </c>
@@ -2102,11 +2115,8 @@
       <c r="M49">
         <v>1.7164600000000001</v>
       </c>
-      <c r="X49">
-        <v>7.3896322613393437</v>
-      </c>
-    </row>
-    <row r="50" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E50">
         <v>5.1141399999999999</v>
       </c>
@@ -2125,11 +2135,8 @@
       <c r="M50">
         <v>1.76261</v>
       </c>
-      <c r="X50">
-        <v>0.70000252109706307</v>
-      </c>
-    </row>
-    <row r="51" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E51">
         <v>5.1612799999999996</v>
       </c>
@@ -2148,11 +2155,8 @@
       <c r="M51">
         <v>1.71648</v>
       </c>
-      <c r="X51">
-        <v>5.3582015232979883</v>
-      </c>
-    </row>
-    <row r="52" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E52">
         <v>5.1025400000000003</v>
       </c>
@@ -2171,11 +2175,8 @@
       <c r="M52">
         <v>1.8131699999999999</v>
       </c>
-      <c r="X52">
-        <v>0.75005655390372228</v>
-      </c>
-    </row>
-    <row r="53" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E53">
         <v>5.1055400000000004</v>
       </c>
@@ -2194,11 +2195,8 @@
       <c r="M53">
         <v>1.7626500000000001</v>
       </c>
-      <c r="X53">
-        <v>3.0017182478681526</v>
-      </c>
-    </row>
-    <row r="54" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E54">
         <v>5.18635</v>
       </c>
@@ -2217,11 +2215,8 @@
       <c r="M54">
         <v>1.7030799999999999</v>
       </c>
-      <c r="X54">
-        <v>0.52247943359597593</v>
-      </c>
-    </row>
-    <row r="55" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E55">
         <v>5.0936300000000001</v>
       </c>
@@ -2240,11 +2235,8 @@
       <c r="M55">
         <v>1.7490000000000001</v>
       </c>
-      <c r="X55">
-        <v>11.680091671013253</v>
-      </c>
-    </row>
-    <row r="56" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E56">
         <v>5.0943199999999997</v>
       </c>
@@ -2263,11 +2255,8 @@
       <c r="M56">
         <v>1.7059800000000001</v>
       </c>
-      <c r="X56">
-        <v>5.0379999999999994</v>
-      </c>
-    </row>
-    <row r="57" spans="5:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E57">
         <v>5.1120700000000001</v>
       </c>
@@ -2287,7 +2276,7 @@
         <v>1.7235100000000001</v>
       </c>
     </row>
-    <row r="58" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="58" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E58">
         <v>5.1306200000000004</v>
       </c>
@@ -2307,7 +2296,7 @@
         <v>1.7233799999999999</v>
       </c>
     </row>
-    <row r="59" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="59" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E59">
         <v>5.1217300000000003</v>
       </c>
@@ -2327,7 +2316,7 @@
         <v>1.8140499999999999</v>
       </c>
     </row>
-    <row r="60" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="60" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E60">
         <v>5.1300400000000002</v>
       </c>
@@ -2341,7 +2330,7 @@
         <v>1.6903300000000001</v>
       </c>
     </row>
-    <row r="61" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="61" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E61">
         <v>5.1863200000000003</v>
       </c>
@@ -2355,7 +2344,7 @@
         <v>1.7617</v>
       </c>
     </row>
-    <row r="62" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="62" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E62">
         <v>5.1861699999999997</v>
       </c>
@@ -2369,7 +2358,7 @@
         <v>1.76142</v>
       </c>
     </row>
-    <row r="63" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="63" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E63">
         <v>5.1885300000000001</v>
       </c>
@@ -2383,7 +2372,7 @@
         <v>1.6284000000000001</v>
       </c>
     </row>
-    <row r="64" spans="5:24" x14ac:dyDescent="0.25">
+    <row r="64" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E64">
         <v>5.1953399999999998</v>
       </c>

</xml_diff>